<commit_message>
feat: implement config loader for CSV, Excel, JSON, and YAML configuration files
</commit_message>
<xml_diff>
--- a/the_energy_company_48100.xlsx
+++ b/the_energy_company_48100.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Shreyas\Documents\Python\Bytehound\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CA4CEE1B-CAB9-4546-AFA6-16E0D8D486BC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FFA3DD00-D2A8-4BE9-965F-D0E0A46EF1DA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="12220" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="409" uniqueCount="167">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="437" uniqueCount="180">
   <si>
     <t>id_or_address</t>
   </si>
@@ -542,6 +542,45 @@
   </si>
   <si>
     <t>max|avg</t>
+  </si>
+  <si>
+    <t>0x1F1</t>
+  </si>
+  <si>
+    <t>BMS_SOC</t>
+  </si>
+  <si>
+    <t>0x1F2</t>
+  </si>
+  <si>
+    <t>BMS_State_Capacity</t>
+  </si>
+  <si>
+    <t>OCV_SOC</t>
+  </si>
+  <si>
+    <t>single</t>
+  </si>
+  <si>
+    <t>%</t>
+  </si>
+  <si>
+    <t>CC_SOC</t>
+  </si>
+  <si>
+    <t>``````</t>
+  </si>
+  <si>
+    <t>SOC</t>
+  </si>
+  <si>
+    <t>State_Capacity</t>
+  </si>
+  <si>
+    <t>Ah</t>
+  </si>
+  <si>
+    <t>Capacity</t>
   </si>
 </sst>
 </file>
@@ -1008,7 +1047,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:F12"/>
+  <dimension ref="A1:F14"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" width="36.1796875" bestFit="1" customWidth="1"/>
@@ -1223,6 +1262,40 @@
         <v>1</v>
       </c>
     </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A13" t="s">
+        <v>167</v>
+      </c>
+      <c r="B13" t="s">
+        <v>168</v>
+      </c>
+      <c r="C13">
+        <v>8</v>
+      </c>
+      <c r="D13" t="s">
+        <v>99</v>
+      </c>
+      <c r="E13" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A14" t="s">
+        <v>169</v>
+      </c>
+      <c r="B14" t="s">
+        <v>170</v>
+      </c>
+      <c r="C14">
+        <v>4</v>
+      </c>
+      <c r="D14" t="s">
+        <v>99</v>
+      </c>
+      <c r="E14" t="b">
+        <v>1</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1230,7 +1303,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:O17"/>
+  <dimension ref="A1:O23"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="13.54296875" bestFit="1" customWidth="1"/>
@@ -1965,6 +2038,125 @@
       </c>
       <c r="N17" t="b">
         <v>1</v>
+      </c>
+    </row>
+    <row r="18" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A18" t="s">
+        <v>167</v>
+      </c>
+      <c r="B18" t="s">
+        <v>171</v>
+      </c>
+      <c r="C18" t="s">
+        <v>172</v>
+      </c>
+      <c r="D18">
+        <v>1</v>
+      </c>
+      <c r="E18" t="s">
+        <v>19</v>
+      </c>
+      <c r="F18">
+        <v>1</v>
+      </c>
+      <c r="G18">
+        <v>0</v>
+      </c>
+      <c r="H18" t="s">
+        <v>173</v>
+      </c>
+      <c r="I18" t="s">
+        <v>176</v>
+      </c>
+      <c r="J18" t="s">
+        <v>23</v>
+      </c>
+      <c r="K18">
+        <v>0</v>
+      </c>
+      <c r="N18" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="19" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A19" t="s">
+        <v>167</v>
+      </c>
+      <c r="B19" t="s">
+        <v>174</v>
+      </c>
+      <c r="C19" t="s">
+        <v>172</v>
+      </c>
+      <c r="D19">
+        <v>1</v>
+      </c>
+      <c r="E19" t="s">
+        <v>19</v>
+      </c>
+      <c r="F19">
+        <v>1</v>
+      </c>
+      <c r="G19">
+        <v>0</v>
+      </c>
+      <c r="H19" t="s">
+        <v>173</v>
+      </c>
+      <c r="I19" t="s">
+        <v>176</v>
+      </c>
+      <c r="J19" t="s">
+        <v>23</v>
+      </c>
+      <c r="K19">
+        <v>0</v>
+      </c>
+      <c r="N19" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="20" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A20" t="s">
+        <v>169</v>
+      </c>
+      <c r="B20" t="s">
+        <v>177</v>
+      </c>
+      <c r="C20" t="s">
+        <v>172</v>
+      </c>
+      <c r="D20">
+        <v>1</v>
+      </c>
+      <c r="E20" t="s">
+        <v>19</v>
+      </c>
+      <c r="F20">
+        <v>1</v>
+      </c>
+      <c r="G20">
+        <v>0</v>
+      </c>
+      <c r="H20" t="s">
+        <v>178</v>
+      </c>
+      <c r="I20" t="s">
+        <v>179</v>
+      </c>
+      <c r="J20" t="s">
+        <v>23</v>
+      </c>
+      <c r="K20">
+        <v>0</v>
+      </c>
+      <c r="N20" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="23" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="L23" t="s">
+        <v>175</v>
       </c>
     </row>
   </sheetData>

</xml_diff>